<commit_message>
Update: spiral dashboard with mass balance, alerts, and optimization
</commit_message>
<xml_diff>
--- a/Spiral Plant Sheet.xlsx
+++ b/Spiral Plant Sheet.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Star\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\spiral analysis attock\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4491AEC-C048-42B0-9C07-6D60975C58B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="2370" windowHeight="0" firstSheet="1" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Spiral Data on Actual Run" sheetId="1" r:id="rId1"/>
@@ -17,7 +18,7 @@
     <sheet name="Sensitivity Analysis Spiral 5" sheetId="3" r:id="rId3"/>
     <sheet name="Feed Flow Distribution Spiral" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -29,10 +30,9 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -624,7 +624,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1240,7 +1240,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1935,7 +1935,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2220,7 +2220,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>